<commit_message>
chore: run 2026-03-22 22:40 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_22_03_2026.xlsx
+++ b/logs/Consolidado_22_03_2026.xlsx
@@ -638,10 +638,10 @@
         <v>152</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
@@ -676,10 +676,10 @@
         <v>78</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -695,10 +695,10 @@
         <v>70</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -714,10 +714,10 @@
         <v>45</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -733,10 +733,10 @@
         <v>104</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>4</v>
@@ -4649,40 +4649,40 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="C97" s="3" t="inlineStr">
         <is>
           <t>Soothing Toning Lotion
 Tónico Suave Hidratante Rosto e Olhos
 200 ml</t>
         </is>
       </c>
-      <c r="D97" s="7" t="inlineStr">
+      <c r="D97" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/soothing-toning-lotion-3001045.html</t>
         </is>
       </c>
-      <c r="E97" s="7" t="inlineStr"/>
-      <c r="F97" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G97" s="7" t="inlineStr">
+      <c r="E97" s="3" t="inlineStr"/>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
         <is>
           <t>3001045</t>
         </is>
       </c>
-      <c r="H97" s="7" t="inlineStr">
+      <c r="H97" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -10930,40 +10930,40 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Spray
 Spray Camomila Aclarador 3-em-1 Cabelo Loiro
 100 ml</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-spray-7615327.html</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>7615327</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -12298,43 +12298,43 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>Mango Nourishing Conditioner
 Condicionador Manga Nutritivo Cabelo Seco</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-conditioner-343975.html</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>5924180</t>
         </is>
       </c>
-      <c r="H50" s="5" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -12384,40 +12384,40 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Mango Nourishing Leave-In Cream
 Creme Dia Manga Nutritivo SOS Cabelo Seco
 125ml</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-leave-in-cream-5072223.html</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>5072223</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -12673,43 +12673,43 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Nettle &amp; Vitamin E Oil Control Dry Shampoo
 Champô Seco Ortiga BIO Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-and-vitamin-e-oil-control-dry-shampoo-366180.html</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>8123735</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H59" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -15081,40 +15081,40 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Head Spa Astera Soothing Freshness &amp; Purity
 Pré-Champô Couro Cabeludo Irritado
 50 ml</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/head-spa-astera-soothing-freshness-and-purity-5520225.html</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>5520225</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -15529,40 +15529,40 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Naturia Invisible Dry Shampoo
 Champô Seco Invisível Lavanda Orgânica
 75 ml</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/naturia-invisible-dry-shampoo-7716350.html</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr"/>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>7716350</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -17901,43 +17901,43 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>7434602</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19876,88 +19876,88 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Giorgio Armani
 Acqua di Gio Eua de Parfum Intense
 Perfume para Homem Amadeirado Fresco</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/acqua-di-gio-eua-de-parfum-intense-446615.html</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>30 ml</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>8697725</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>45%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Giorgio Armani
 Acqua di Gio Eua de Parfum Intense
 Perfume para Homem Amadeirado Fresco</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/acqua-di-gio-eua-de-parfum-intense-446615.html</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>8697727</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>45%</t>
         </is>
@@ -23800,17 +23800,17 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="inlineStr">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
+      <c r="C99" s="7" t="inlineStr">
         <is>
           <t>L'Oréal Paris
 Revitalift Glass Skin Creme Líquido
@@ -23818,23 +23818,23 @@
 50 ml</t>
         </is>
       </c>
-      <c r="D99" s="5" t="inlineStr">
+      <c r="D99" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/revitalift-glass-skin-creme-liquido-8684540.html</t>
         </is>
       </c>
-      <c r="E99" s="5" t="inlineStr"/>
-      <c r="F99" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
+      <c r="E99" s="7" t="inlineStr"/>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
         <is>
           <t>8684540</t>
         </is>
       </c>
-      <c r="H99" s="5" t="inlineStr">
+      <c r="H99" s="7" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -24904,38 +24904,38 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>7434602</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
@@ -27257,38 +27257,38 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="7" t="inlineStr">
         <is>
           <t>Mango Nourishing Conditioner
 Condicionador Manga Nutritivo Cabelo Seco</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
         <is>
           <t>5924180</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G66" s="3" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-conditioner-343975.html</t>
         </is>
@@ -27485,38 +27485,38 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Nettle &amp; Vitamin E Oil Control Dry Shampoo
 Champô Seco Ortiga BIO Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>8123735</t>
         </is>
       </c>
-      <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-and-vitamin-e-oil-control-dry-shampoo-366180.html</t>
         </is>
@@ -28170,78 +28170,78 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>Giorgio Armani
 Acqua di Gio Eua de Parfum Intense
 Perfume para Homem Amadeirado Fresco</t>
         </is>
       </c>
-      <c r="C90" s="3" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>30 ml</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E90" s="3" t="inlineStr">
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
         <is>
           <t>8697725</t>
         </is>
       </c>
-      <c r="F90" s="3" t="inlineStr">
+      <c r="F90" s="7" t="inlineStr">
         <is>
           <t>45%</t>
         </is>
       </c>
-      <c r="G90" s="3" t="inlineStr">
+      <c r="G90" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/acqua-di-gio-eua-de-parfum-intense-446615.html</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="3" t="inlineStr">
+      <c r="A91" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B91" s="7" t="inlineStr">
         <is>
           <t>Giorgio Armani
 Acqua di Gio Eua de Parfum Intense
 Perfume para Homem Amadeirado Fresco</t>
         </is>
       </c>
-      <c r="C91" s="3" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E91" s="3" t="inlineStr">
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
         <is>
           <t>8697727</t>
         </is>
       </c>
-      <c r="F91" s="3" t="inlineStr">
+      <c r="F91" s="7" t="inlineStr">
         <is>
           <t>45%</t>
         </is>
       </c>
-      <c r="G91" s="3" t="inlineStr">
+      <c r="G91" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/acqua-di-gio-eua-de-parfum-intense-446615.html</t>
         </is>

</xml_diff>